<commit_message>
Done with day 42
</commit_message>
<xml_diff>
--- a/2.Patterns Practice.xlsx
+++ b/2.Patterns Practice.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="563" uniqueCount="244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="564" uniqueCount="244">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -2267,7 +2267,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="22" t="n">
         <v>1</v>
       </c>
@@ -2290,7 +2290,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="22" t="n">
         <v>2</v>
       </c>
@@ -2313,7 +2313,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="22" t="n">
         <v>3</v>
       </c>
@@ -2336,7 +2336,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="26" t="n">
         <v>4</v>
       </c>
@@ -2359,7 +2359,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="22" t="n">
         <v>5</v>
       </c>
@@ -2382,7 +2382,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="22" t="n">
         <v>6</v>
       </c>
@@ -2405,7 +2405,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="22" t="n">
         <v>7</v>
       </c>
@@ -2428,7 +2428,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="30" t="n">
         <v>8</v>
       </c>
@@ -2451,7 +2451,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="22" t="n">
         <v>9</v>
       </c>
@@ -2474,7 +2474,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="22" t="n">
         <v>10</v>
       </c>
@@ -2497,7 +2497,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="22" t="n">
         <v>11</v>
       </c>
@@ -18578,7 +18578,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="69" width="69.19"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="6" min="6" style="69" width="11.55"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="69" width="10.4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="75" width="44.23"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="75" width="44.24"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="9" style="69" width="11.55"/>
   </cols>
   <sheetData>
@@ -18641,6 +18641,9 @@
       <c r="E3" s="75" t="s">
         <v>218</v>
       </c>
+      <c r="G3" s="69" t="n">
+        <v>42</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="75" t="n">
@@ -18693,7 +18696,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="37.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="75" t="n">
         <v>6</v>
       </c>
@@ -18768,6 +18771,12 @@
       </c>
       <c r="E10" s="75" t="s">
         <v>234</v>
+      </c>
+      <c r="F10" s="69" t="s">
+        <v>11</v>
+      </c>
+      <c r="G10" s="69" t="n">
+        <v>42</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Done with day 43
</commit_message>
<xml_diff>
--- a/2.Patterns Practice.xlsx
+++ b/2.Patterns Practice.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="564" uniqueCount="244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="568" uniqueCount="246">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -686,6 +686,9 @@
     <t xml:space="preserve">https://leetcode.com/problems/find-median-from-data-stream/</t>
   </si>
   <si>
+    <t xml:space="preserve">Practice 2 heaps(max-min) to find median</t>
+  </si>
+  <si>
     <t xml:space="preserve">480. Sliding Window Median</t>
   </si>
   <si>
@@ -744,6 +747,9 @@
   </si>
   <si>
     <t xml:space="preserve">https://leetcode.com/problems/the-number-of-the-smallest-unoccupied-chair/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Base problem - Many similar problems revolve around this pattern</t>
   </si>
   <si>
     <t xml:space="preserve">1354. Construct Target Array With Multiple Sums</t>
@@ -769,7 +775,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0"/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="25">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -935,6 +941,21 @@
       <family val="4"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Comic Sans MS"/>
+      <family val="4"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Comic Sans MS"/>
+      <family val="4"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -1062,7 +1083,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="79">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1363,12 +1384,20 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="24" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="24" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -2267,7 +2296,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="22" t="n">
         <v>1</v>
       </c>
@@ -2290,7 +2319,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="22" t="n">
         <v>2</v>
       </c>
@@ -2313,7 +2342,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="22" t="n">
         <v>3</v>
       </c>
@@ -2336,7 +2365,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="26" t="n">
         <v>4</v>
       </c>
@@ -2359,7 +2388,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="22" t="n">
         <v>5</v>
       </c>
@@ -2382,7 +2411,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="22" t="n">
         <v>6</v>
       </c>
@@ -2405,7 +2434,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="22" t="n">
         <v>7</v>
       </c>
@@ -2428,7 +2457,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="30" t="n">
         <v>8</v>
       </c>
@@ -2451,7 +2480,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="22" t="n">
         <v>9</v>
       </c>
@@ -2474,7 +2503,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="22" t="n">
         <v>10</v>
       </c>
@@ -2497,7 +2526,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="22" t="n">
         <v>11</v>
       </c>
@@ -18132,8 +18161,8 @@
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
@@ -18557,8 +18586,8 @@
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
@@ -18571,303 +18600,318 @@
   <dimension ref="A1:H15"/>
   <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="16.15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="69" width="5.31"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="2" min="2" style="69" width="11.55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="69" width="64.07"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="69" width="19.77"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="69" width="69.19"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="6" min="6" style="69" width="11.55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="69" width="10.4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="75" width="44.24"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="9" style="69" width="11.55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="75" width="5.31"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="2" min="2" style="75" width="11.55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="75" width="64.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="75" width="19.77"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="75" width="69.19"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="6" min="6" style="75" width="11.55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="75" width="10.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="76" width="77.76"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="9" style="75" width="11.55"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="76" t="s">
+    <row r="1" customFormat="false" ht="18.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="77" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="76" t="s">
+      <c r="B1" s="77" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="76" t="s">
+      <c r="C1" s="77" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="76" t="s">
+      <c r="D1" s="77" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="76" t="s">
+      <c r="E1" s="77" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="76" t="s">
+      <c r="F1" s="77" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="71" t="s">
+      <c r="G1" s="78" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="71" t="s">
+      <c r="H1" s="78" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="75" t="n">
+    <row r="2" customFormat="false" ht="18.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="76" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="75" t="s">
+      <c r="B2" s="76" t="s">
         <v>214</v>
       </c>
-      <c r="C2" s="75" t="s">
+      <c r="C2" s="76" t="s">
         <v>215</v>
       </c>
-      <c r="D2" s="75" t="s">
+      <c r="D2" s="76" t="s">
         <v>34</v>
       </c>
-      <c r="E2" s="75" t="s">
+      <c r="E2" s="76" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="75" t="n">
+    <row r="3" customFormat="false" ht="18.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="76" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="75" t="s">
+      <c r="B3" s="76" t="s">
         <v>214</v>
       </c>
-      <c r="C3" s="75" t="s">
+      <c r="C3" s="76" t="s">
         <v>217</v>
       </c>
-      <c r="D3" s="75" t="s">
+      <c r="D3" s="76" t="s">
         <v>34</v>
       </c>
-      <c r="E3" s="75" t="s">
+      <c r="E3" s="76" t="s">
         <v>218</v>
       </c>
-      <c r="G3" s="69" t="n">
+      <c r="F3" s="75" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3" s="75" t="n">
         <v>42</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="75" t="n">
+      <c r="H3" s="76" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="18.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="76" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="75" t="s">
+      <c r="B4" s="76" t="s">
         <v>214</v>
       </c>
-      <c r="C4" s="75" t="s">
-        <v>219</v>
-      </c>
-      <c r="D4" s="75" t="s">
+      <c r="C4" s="76" t="s">
         <v>220</v>
       </c>
-      <c r="E4" s="75" t="s">
+      <c r="D4" s="76" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="75" t="n">
+      <c r="E4" s="76" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="18.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="76" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="75" t="s">
+      <c r="B5" s="76" t="s">
         <v>214</v>
       </c>
-      <c r="C5" s="75" t="s">
+      <c r="C5" s="76" t="s">
+        <v>223</v>
+      </c>
+      <c r="D5" s="76" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" s="76" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="18.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="76" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="76" t="s">
+        <v>214</v>
+      </c>
+      <c r="C6" s="76" t="s">
+        <v>225</v>
+      </c>
+      <c r="D6" s="76" t="s">
+        <v>34</v>
+      </c>
+      <c r="E6" s="76" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="34.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="76" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="76" t="s">
+        <v>214</v>
+      </c>
+      <c r="C7" s="76" t="s">
+        <v>227</v>
+      </c>
+      <c r="D7" s="76" t="s">
+        <v>9</v>
+      </c>
+      <c r="E7" s="76" t="s">
+        <v>228</v>
+      </c>
+      <c r="F7" s="75" t="s">
+        <v>11</v>
+      </c>
+      <c r="G7" s="75" t="n">
+        <v>41</v>
+      </c>
+      <c r="H7" s="76" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="18.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="76" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="76" t="s">
+        <v>214</v>
+      </c>
+      <c r="C8" s="76" t="s">
+        <v>230</v>
+      </c>
+      <c r="D8" s="76" t="s">
+        <v>19</v>
+      </c>
+      <c r="E8" s="76" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="18.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="76" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="76" t="s">
+        <v>214</v>
+      </c>
+      <c r="C9" s="76" t="s">
+        <v>232</v>
+      </c>
+      <c r="D9" s="76" t="s">
+        <v>19</v>
+      </c>
+      <c r="E9" s="76" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="18.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="76" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="76" t="s">
+        <v>214</v>
+      </c>
+      <c r="C10" s="76" t="s">
+        <v>234</v>
+      </c>
+      <c r="D10" s="76" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10" s="76" t="s">
+        <v>235</v>
+      </c>
+      <c r="F10" s="75" t="s">
+        <v>11</v>
+      </c>
+      <c r="G10" s="75" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="18.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="76" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="76" t="s">
+        <v>214</v>
+      </c>
+      <c r="C11" s="76" t="s">
+        <v>236</v>
+      </c>
+      <c r="D11" s="76" t="s">
+        <v>19</v>
+      </c>
+      <c r="E11" s="76" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="18.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="76" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="76" t="s">
+        <v>214</v>
+      </c>
+      <c r="C12" s="76" t="s">
+        <v>238</v>
+      </c>
+      <c r="D12" s="76" t="s">
+        <v>19</v>
+      </c>
+      <c r="E12" s="76" t="s">
+        <v>239</v>
+      </c>
+      <c r="F12" s="75" t="s">
+        <v>11</v>
+      </c>
+      <c r="G12" s="75" t="n">
+        <v>43</v>
+      </c>
+      <c r="H12" s="76" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="18.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="76" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="76" t="s">
+        <v>214</v>
+      </c>
+      <c r="C13" s="76" t="s">
+        <v>241</v>
+      </c>
+      <c r="D13" s="76" t="s">
+        <v>34</v>
+      </c>
+      <c r="E13" s="76" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="18.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="76" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="76" t="s">
+        <v>214</v>
+      </c>
+      <c r="C14" s="76" t="s">
+        <v>243</v>
+      </c>
+      <c r="D14" s="76" t="s">
+        <v>9</v>
+      </c>
+      <c r="E14" s="76" t="s">
+        <v>244</v>
+      </c>
+      <c r="F14" s="75" t="s">
+        <v>11</v>
+      </c>
+      <c r="G14" s="75" t="n">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="18.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="76" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="76" t="s">
+        <v>214</v>
+      </c>
+      <c r="C15" s="76" t="s">
+        <v>220</v>
+      </c>
+      <c r="D15" s="76" t="s">
+        <v>245</v>
+      </c>
+      <c r="E15" s="76" t="s">
         <v>222</v>
-      </c>
-      <c r="D5" s="75" t="s">
-        <v>19</v>
-      </c>
-      <c r="E5" s="75" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="75" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="75" t="s">
-        <v>214</v>
-      </c>
-      <c r="C6" s="75" t="s">
-        <v>224</v>
-      </c>
-      <c r="D6" s="75" t="s">
-        <v>34</v>
-      </c>
-      <c r="E6" s="75" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="75" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="75" t="s">
-        <v>214</v>
-      </c>
-      <c r="C7" s="75" t="s">
-        <v>226</v>
-      </c>
-      <c r="D7" s="75" t="s">
-        <v>9</v>
-      </c>
-      <c r="E7" s="75" t="s">
-        <v>227</v>
-      </c>
-      <c r="F7" s="69" t="s">
-        <v>11</v>
-      </c>
-      <c r="G7" s="69" t="n">
-        <v>41</v>
-      </c>
-      <c r="H7" s="75" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="75" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="75" t="s">
-        <v>214</v>
-      </c>
-      <c r="C8" s="75" t="s">
-        <v>229</v>
-      </c>
-      <c r="D8" s="75" t="s">
-        <v>19</v>
-      </c>
-      <c r="E8" s="75" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="75" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="75" t="s">
-        <v>214</v>
-      </c>
-      <c r="C9" s="75" t="s">
-        <v>231</v>
-      </c>
-      <c r="D9" s="75" t="s">
-        <v>19</v>
-      </c>
-      <c r="E9" s="75" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="75" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="75" t="s">
-        <v>214</v>
-      </c>
-      <c r="C10" s="75" t="s">
-        <v>233</v>
-      </c>
-      <c r="D10" s="75" t="s">
-        <v>19</v>
-      </c>
-      <c r="E10" s="75" t="s">
-        <v>234</v>
-      </c>
-      <c r="F10" s="69" t="s">
-        <v>11</v>
-      </c>
-      <c r="G10" s="69" t="n">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="75" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="75" t="s">
-        <v>214</v>
-      </c>
-      <c r="C11" s="75" t="s">
-        <v>235</v>
-      </c>
-      <c r="D11" s="75" t="s">
-        <v>19</v>
-      </c>
-      <c r="E11" s="75" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="75" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" s="75" t="s">
-        <v>214</v>
-      </c>
-      <c r="C12" s="75" t="s">
-        <v>237</v>
-      </c>
-      <c r="D12" s="75" t="s">
-        <v>19</v>
-      </c>
-      <c r="E12" s="75" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="75" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" s="75" t="s">
-        <v>214</v>
-      </c>
-      <c r="C13" s="75" t="s">
-        <v>239</v>
-      </c>
-      <c r="D13" s="75" t="s">
-        <v>34</v>
-      </c>
-      <c r="E13" s="75" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="75" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" s="75" t="s">
-        <v>214</v>
-      </c>
-      <c r="C14" s="75" t="s">
-        <v>241</v>
-      </c>
-      <c r="D14" s="75" t="s">
-        <v>9</v>
-      </c>
-      <c r="E14" s="75" t="s">
-        <v>242</v>
-      </c>
-      <c r="F14" s="69" t="s">
-        <v>11</v>
-      </c>
-      <c r="G14" s="69" t="n">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="75" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" s="75" t="s">
-        <v>214</v>
-      </c>
-      <c r="C15" s="75" t="s">
-        <v>219</v>
-      </c>
-      <c r="D15" s="75" t="s">
-        <v>243</v>
-      </c>
-      <c r="E15" s="75" t="s">
-        <v>221</v>
       </c>
     </row>
   </sheetData>
@@ -18891,8 +18935,8 @@
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Done with day 44
</commit_message>
<xml_diff>
--- a/2.Patterns Practice.xlsx
+++ b/2.Patterns Practice.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="568" uniqueCount="246">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="570" uniqueCount="247">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -708,6 +708,27 @@
   </si>
   <si>
     <t xml:space="preserve">https://leetcode.com/problems/meeting-rooms-iii/</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Comic Sans MS"/>
+        <family val="4"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Solve this and Leetcode </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Comic Sans MS"/>
+        <family val="4"/>
+      </rPr>
+      <t xml:space="preserve">1942 together</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">2231. Largest Number After Digit Swaps by Parity</t>
@@ -775,7 +796,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0"/>
   </numFmts>
-  <fonts count="25">
+  <fonts count="26">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -955,6 +976,12 @@
       <name val="Comic Sans MS"/>
       <family val="4"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Comic Sans MS"/>
+      <family val="4"/>
     </font>
   </fonts>
   <fills count="8">
@@ -2296,7 +2323,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="22" t="n">
         <v>1</v>
       </c>
@@ -2319,7 +2346,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="22" t="n">
         <v>2</v>
       </c>
@@ -2342,7 +2369,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="22" t="n">
         <v>3</v>
       </c>
@@ -2365,7 +2392,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="26" t="n">
         <v>4</v>
       </c>
@@ -2388,7 +2415,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="22" t="n">
         <v>5</v>
       </c>
@@ -2411,7 +2438,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="22" t="n">
         <v>6</v>
       </c>
@@ -2434,7 +2461,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="22" t="n">
         <v>7</v>
       </c>
@@ -2457,7 +2484,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="30" t="n">
         <v>8</v>
       </c>
@@ -2480,7 +2507,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="22" t="n">
         <v>9</v>
       </c>
@@ -2503,7 +2530,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="22" t="n">
         <v>10</v>
       </c>
@@ -2526,7 +2553,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="22" t="n">
         <v>11</v>
       </c>
@@ -18730,8 +18757,17 @@
       <c r="E6" s="76" t="s">
         <v>226</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="34.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F6" s="75" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6" s="75" t="n">
+        <v>44</v>
+      </c>
+      <c r="H6" s="76" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="35.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="76" t="n">
         <v>6</v>
       </c>
@@ -18739,13 +18775,13 @@
         <v>214</v>
       </c>
       <c r="C7" s="76" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="D7" s="76" t="s">
         <v>9</v>
       </c>
       <c r="E7" s="76" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="F7" s="75" t="s">
         <v>11</v>
@@ -18754,7 +18790,7 @@
         <v>41</v>
       </c>
       <c r="H7" s="76" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="18.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18765,13 +18801,13 @@
         <v>214</v>
       </c>
       <c r="C8" s="76" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D8" s="76" t="s">
         <v>19</v>
       </c>
       <c r="E8" s="76" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="18.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18782,13 +18818,13 @@
         <v>214</v>
       </c>
       <c r="C9" s="76" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="D9" s="76" t="s">
         <v>19</v>
       </c>
       <c r="E9" s="76" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="18.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18799,13 +18835,13 @@
         <v>214</v>
       </c>
       <c r="C10" s="76" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D10" s="76" t="s">
         <v>19</v>
       </c>
       <c r="E10" s="76" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="F10" s="75" t="s">
         <v>11</v>
@@ -18822,13 +18858,13 @@
         <v>214</v>
       </c>
       <c r="C11" s="76" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="D11" s="76" t="s">
         <v>19</v>
       </c>
       <c r="E11" s="76" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="18.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18839,13 +18875,13 @@
         <v>214</v>
       </c>
       <c r="C12" s="76" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="D12" s="76" t="s">
         <v>19</v>
       </c>
       <c r="E12" s="76" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="F12" s="75" t="s">
         <v>11</v>
@@ -18854,7 +18890,7 @@
         <v>43</v>
       </c>
       <c r="H12" s="76" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="18.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18865,13 +18901,13 @@
         <v>214</v>
       </c>
       <c r="C13" s="76" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D13" s="76" t="s">
         <v>34</v>
       </c>
       <c r="E13" s="76" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="18.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18882,13 +18918,13 @@
         <v>214</v>
       </c>
       <c r="C14" s="76" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D14" s="76" t="s">
         <v>9</v>
       </c>
       <c r="E14" s="76" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="F14" s="75" t="s">
         <v>11</v>
@@ -18908,7 +18944,7 @@
         <v>220</v>
       </c>
       <c r="D15" s="76" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="E15" s="76" t="s">
         <v>222</v>

</xml_diff>

<commit_message>
Binary Tree Maximum Path Sum
</commit_message>
<xml_diff>
--- a/2.Patterns Practice.xlsx
+++ b/2.Patterns Practice.xlsx
@@ -710,25 +710,7 @@
     <t xml:space="preserve">https://leetcode.com/problems/meeting-rooms-iii/</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Comic Sans MS"/>
-        <family val="4"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Solve this and Leetcode </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Comic Sans MS"/>
-        <family val="4"/>
-      </rPr>
-      <t xml:space="preserve">1942 together</t>
-    </r>
+    <t xml:space="preserve">Solve this and Leetcode 1942 together</t>
   </si>
   <si>
     <t xml:space="preserve">2231. Largest Number After Digit Swaps by Parity</t>
@@ -796,7 +778,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0"/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="25">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -976,12 +958,6 @@
       <name val="Comic Sans MS"/>
       <family val="4"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Comic Sans MS"/>
-      <family val="4"/>
     </font>
   </fonts>
   <fills count="8">
@@ -2323,7 +2299,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="22" t="n">
         <v>1</v>
       </c>
@@ -2346,7 +2322,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="22" t="n">
         <v>2</v>
       </c>
@@ -2369,7 +2345,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="22" t="n">
         <v>3</v>
       </c>
@@ -2392,7 +2368,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="26" t="n">
         <v>4</v>
       </c>
@@ -2415,7 +2391,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="22" t="n">
         <v>5</v>
       </c>
@@ -2438,7 +2414,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="22" t="n">
         <v>6</v>
       </c>
@@ -2461,7 +2437,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="22" t="n">
         <v>7</v>
       </c>
@@ -2484,7 +2460,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="30" t="n">
         <v>8</v>
       </c>
@@ -2507,7 +2483,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="22" t="n">
         <v>9</v>
       </c>
@@ -2530,7 +2506,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="22" t="n">
         <v>10</v>
       </c>
@@ -2553,7 +2529,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="22" t="n">
         <v>11</v>
       </c>

</xml_diff>